<commit_message>
chore(toy): stamp the build on the sheet — three rounds were spent on an already-fixed defect
The grower, on an already-corrected annual cap: "The v5 still has the wrong demand cap for
kale." The file on disk was right; the copy open on their machine was not. The filename never
changes between rebuilds, so there has been no way to tell one build from the next, and this is
the third round lost to it.

Model!D1 and READ ME row 2 now carry the build time and the commit short-sha, so a version can
be confirmed at a glance instead of by re-deriving a formula.

Verified on this build: the Kale/Wholesale ceiling formula is $D$21-SUM(E146:AG146), row 146 is
that pair's SOLD row, and once solved the allowance declines 500,000 -> 473,886 -> 442,579 ->
389,448 -> 162,472 across weeks 1/20/30/40/52.

433 pytest + toy verifier green.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAF5GH3ATcx4Hk54BqMfPb
</commit_message>
<xml_diff>
--- a/toy_models/farm_toy_v5_full_calendar.xlsx
+++ b/toy_models/farm_toy_v5_full_calendar.xlsx
@@ -140,9 +140,9 @@
   <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A136"/>
+  <dimension ref="A1:A139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="112" customWidth="1" min="1" max="1"/>
@@ -588,463 +588,467 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>BUILT 2026-08-30 13:25   (from source at commit a6c69e1)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>If that timestamp is older than the change you are looking for, you have a stale copy —</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>close the file and re-open it from WSL rather than from a recent-files list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
           <t>WHAT v5 ADDS — both of these you spotted missing from v4</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>1. IT CHOOSES WHEN TO PLANT.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t xml:space="preserve">   All 68 plantings the app's calendar generator offers are on the sheet, one row per legal</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t xml:space="preserve">   start week. The solver puts acres on some and zero on others — and zero acres IS the</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   decision not to plant that week. v4 offered five that I picked by hand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>2. IT CHOOSES WHETHER TO PLANT AT ALL.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   The BLUE column is a binary per planting, tied to the acres by two constraints that are</t>
+          <t xml:space="preserve">   decision not to plant that week. v4 offered five that I picked by hand.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   the app's own C9 and C10:</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        acres &lt;= 'max if planted'   you cannot plant acres without deciding to plant</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2. IT CHOOSES WHETHER TO PLANT AT ALL.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">        acres &gt;= 'min if planted'   if you plant at all, you plant a real block</t>
+          <t xml:space="preserve">   The BLUE column is a binary per planting, tied to the acres by two constraints that are</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   That is what stops it planting a third of an acre, and it makes this a MILP — which is</t>
+          <t xml:space="preserve">   the app's own C9 and C10:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   what farm_v2/solver.py is. Its `integrality` array marks the very same y block.</t>
+          <t xml:space="preserve">        acres &lt;= 'max if planted'   you cannot plant acres without deciding to plant</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        acres &gt;= 'min if planted'   if you plant at all, you plant a real block</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>WHAT THE TWO CHANGES ARE WORTH — measured, and they pull OPPOSITE ways</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   That is what stops it planting a third of an acre, and it makes this a MILP — which is</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">     v4, five hand-picked plantings          $1,094,831</t>
+          <t xml:space="preserve">   what farm_v2/solver.py is. Its `integrality` array marks the very same y block.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     v5 without the minimum-acreage rule     $2,387,990   (42 plantings)</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">     v5 as it ships                          $2,384,231   (33 plantings)</t>
+          <t>WHAT THE TWO CHANGES ARE WORTH — measured, and they pull OPPOSITE ways</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     v4, five hand-picked plantings          $1,094,831</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t xml:space="preserve">     v5 without the minimum-acreage rule     $2,387,990   (42 plantings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     v5 as it ships                          $2,384,231   (33 plantings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Letting it choose the weeks more than doubles profit. Then the minimum-acreage rule takes</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>$3,759 back and drops the plan from 42 plantings to 33, because the</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>slivers are gone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Neither number means anything alone. A fixed calendar UNDERSTATES; a missing minimum</t>
+          <t>$3,759 back and drops the plan from 42 plantings to 33, because the</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>slivers are gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Neither number means anything alone. A fixed calendar UNDERSTATES; a missing minimum</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>acreage OVERSTATES. That is why the real model has both, and it is the reason it is a MILP</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>rather than a plain LP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>WHY IT PLANTS SO MANY — this is the finding worth keeping</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>33 plantings out of 68, staggered across the season rather than a few big</t>
+          <t>rather than a plain LP.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>blocks. That is SUCCESSION PLANTING, and now you can see why it pays: spreading the harvest</t>
-        </is>
-      </c>
+      <c r="A33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>is what lets you serve a WEEKLY demand cap continuously. Plant it all at once and one huge</t>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>WHY IT PLANTS SO MANY — this is the finding worth keeping</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>harvest slams into the ceiling, the cooler fills, and the surplus is wasted or dumped cheap.</t>
+          <t>33 plantings out of 68, staggered across the season rather than a few big</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>blocks. That is SUCCESSION PLANTING, and now you can see why it pays: spreading the harvest</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>A model with a fixed planting calendar cannot express the thing the practice exists for.</t>
+          <t>is what lets you serve a WEEKLY demand cap continuously. Plant it all at once and one huge</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>harvest slams into the ceiling, the cooler fills, and the surplus is wasted or dumped cheap.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>!! IT NEEDS LIBREOFFICE, AND THIS ONE IS A REAL MILP</t>
-        </is>
-      </c>
+      <c r="A39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>A model with a fixed planting calendar cannot express the thing the practice exists for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>!! IT NEEDS LIBREOFFICE, AND THIS ONE IS A REAL MILP</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>448 decision cells: 68 acres + 68 binaries + 312 offered. The engine MUST be</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>CoinMP — it does branch and bound over the integers. Expect it to take appreciably longer</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>than v4; integers are what make an optimizer work for its living.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>WHERE THINGS ARE</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  YELLOW   you type: the farm, the crop table, the crop x channel table.</t>
+          <t>than v4; integers are what make an optimizer work for its living.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  GREEN    the solver writes: the ACRES column (C28:C95), the six OFFERED rows, and</t>
-        </is>
-      </c>
+      <c r="A46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">           the PROFIT cell (B200).</t>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>WHERE THINGS ARE</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  BLUE     the solver writes: the PLANT? binaries (D28:D95).</t>
+          <t xml:space="preserve">  YELLOW   you type: the farm, the crop table, the crop x channel table.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Everything else is a formula. Columns A-D stay put when you scroll right.</t>
+          <t xml:space="preserve">  GREEN    the solver writes: the ACRES column (C28:C95), the six OFFERED rows, and</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           the PROFIT cell (B200).</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>HOW TO RUN IT</t>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  BLUE     the solver writes: the PLANT? binaries (D28:D95).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Section 7 lists every entry with exact ranges. In short:</t>
+          <t xml:space="preserve">  Everything else is a formula. Columns A-D stay put when you scroll right.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Tools &gt; Solver, target the PROFIT cell, set to MAXIMUM</t>
-        </is>
-      </c>
+      <c r="A53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Changing cells: C28:C95 and D28:D95 together, plus the six OFFERED rows</t>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO RUN IT</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Add the constraint  D28:D95 = Binary   — without it the binaries are just numbers</t>
+          <t>Section 7 lists every entry with exact ranges. In short:</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   and the minimum-acreage rule silently stops working</t>
+          <t xml:space="preserve">   Tools &gt; Solver, target the PROFIT cell, set to MAXIMUM</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Changing cells: C28:C95 and D28:D95 together, plus the six OFFERED rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Add the constraint  D28:D95 = Binary   — without it the binaries are just numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   and the minimum-acreage rule silently stops working</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Options: engine = LibreOffice CoinMP Linear Solver; tick non-negative</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>WHAT IT SHOULD FIND</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">     PROFIT   $2,384,231      = revenue $2,558,846 - growing cost $174,616</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">     33 of 68 plantings used</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>Computed by solving the same MILP with scipy.milp — the same HiGHS solver your app runs. A</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>few dollars apart is tolerances. Materially different means one of the two models is not the</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>model we think it is.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>WHAT SELL-THROUGH IS, AND WHY IT SHIPS AT 1.00</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Every 'Sell-through' in section 3 is 1.00, matching the app since 30 Aug. The 85% it used to</t>
+          <t>model we think it is.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>carry had no source, and it was being charged on channels where a purchase order exists and</t>
-        </is>
-      </c>
+      <c r="A69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>nothing goes unsold. So the market-loss and returned-to-store rows all read ZERO right now.</t>
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>WHAT SELL-THROUGH IS, AND WHY IT SHIPS AT 1.00</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>That is correct, not broken.</t>
+          <t>Every 'Sell-through' in section 3 is 1.00, matching the app since 30 Aug. The 85% it used to</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>carry had no source, and it was being charged on channels where a purchase order exists and</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>nothing goes unsold. So the market-loss and returned-to-store rows all read ZERO right now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>That is correct, not broken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
           <t>The narrow definition it now carries:</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Of what you TAKE TO MARKET, the share that converts to cash — display attrition at a</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     stall, samples, transit damage, a rejected load.</t>
         </is>
       </c>
     </row>
@@ -1052,377 +1056,394 @@
       <c r="A77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Of what you TAKE TO MARKET, the share that converts to cash — display attrition at a</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     stall, samples, transit damage, a rejected load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
         <is>
           <t>NOT grade-out at harvest (that is pack-out, above the store). NOT spoilage in the store (that</t>
         </is>
       </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>is shrink). And NOT demand uncertainty — which is the one worth understanding, because it is</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>why the old wording could not be right:</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">     The demand ceiling is HARD. At a 6,000 lb cap and 0.85, selling 6,000 means bringing</t>
+          <t>is shrink). And NOT demand uncertainty — which is the one worth understanding, because it is</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">     7,059 and losing 1,059 — every week, including the best Saturday of the year, because</t>
+          <t>why the old wording could not be right:</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     the model will never let you sell 6,001. That is the whole downside of bringing extra</t>
-        </is>
-      </c>
+      <c r="A84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">     with none of the upside. It is not a model of uncertainty; it is a one-sided penalty.</t>
+          <t xml:space="preserve">     The demand ceiling is HARD. At a 6,000 lb cap and 0.85, selling 6,000 means bringing</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     7,059 and losing 1,059 — every week, including the best Saturday of the year, because</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>So what it CAN mean is a display requirement: a picked-over stall sells less than a full one,</t>
+          <t xml:space="preserve">     the model will never let you sell 6,001. That is the whole downside of bringing extra</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>so moving 6,000 lb needs more than 6,000 lb on the table. Deterministic, and an input</t>
+          <t xml:space="preserve">     with none of the upside. It is not a model of uncertainty; it is a one-sided penalty.</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>requirement like seed. Real demand variance is a different problem (newsvendor) needing</t>
-        </is>
-      </c>
+      <c r="A89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>So what it CAN mean is a display requirement: a picked-over stall sells less than a full one,</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>so moving 6,000 lb needs more than 6,000 lb on the table. Deterministic, and an input</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>requirement like seed. Real demand variance is a different problem (newsvendor) needing</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
           <t>machinery neither this sheet nor the app has yet.</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>THREE THINGS TO TRY</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr"/>
-    </row>
     <row r="94">
-      <c r="A94" s="3" t="inlineStr">
-        <is>
-          <t>EXPERIMENT 1 — switch sell-through on, and watch the crop decide what happens.</t>
-        </is>
-      </c>
+      <c r="A94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
+          <t>THREE THINGS TO TRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>EXPERIMENT 1 — switch sell-through on, and watch the crop decide what happens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">   In section 3 set Spinach / {CH1} sell-through to 0.85, and Garlic / {CH1} to 0.85 too.</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="3" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   Re-solve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Both now offer more than they sell. But look at the two 'market loss' rows: Spinach's is</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   positive and Garlic's is ZERO, because garlic's 'Returns to store' is 1.00 — unsold garlic</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   comes home and sells later, so the loss is a DELAY, not a loss.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">   That is the grower's ruling in two cells: the same sell-through means different things on</t>
+          <t xml:space="preserve">   Both now offer more than they sell. But look at the two 'market loss' rows: Spinach's is</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">   different crops, which is why it belongs on the crop x channel row and not on either one</t>
+          <t xml:space="preserve">   positive and Garlic's is ZERO, because garlic's 'Returns to store' is 1.00 — unsold garlic</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">   alone. Now set Garlic's 'Returns to store' to 0.00 and re-solve: the delay becomes a loss</t>
+          <t xml:space="preserve">   comes home and sells later, so the loss is a DELAY, not a loss.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t xml:space="preserve">   That is the grower's ruling in two cells: the same sell-through means different things on</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   different crops, which is why it belongs on the crop x channel row and not on either one</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   alone. Now set Garlic's 'Returns to store' to 0.00 and re-solve: the delay becomes a loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
           <t xml:space="preserve">   and the plan changes.</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="3" t="inlineStr">
+    <row r="107">
+      <c r="A107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
         <is>
           <t>EXPERIMENT 2 — drop the minimum acreage.  Set every 'Min acres if planted' in the crop</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="3" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   table to 0 and re-solve.</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
+    <row r="110">
+      <c r="A110" t="inlineStr">
         <is>
           <t xml:space="preserve">   Expect $2,387,990 and 42 plantings. The extra profit is real but the plan is</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
+    <row r="111">
+      <c r="A111" t="inlineStr">
         <is>
           <t xml:space="preserve">   not: it plants fractions of an acre no one would drive a tractor out for. This is what</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   the binaries are FOR, and it is why the app carries them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="3" t="inlineStr">
-        <is>
-          <t>EXPERIMENT 3 — take away the cooler.  Set the cold store to 40 m3 and re-solve.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
+          <t xml:space="preserve">   the binaries are FOR, and it is why the app carries them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>EXPERIMENT 3 — take away the cooler.  Set the cold store to 40 m3 and re-solve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Watch WHICH WEEKS it abandons, not just which crop. With a full calendar it can retreat</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
+    <row r="116">
+      <c r="A116" t="inlineStr">
         <is>
           <t xml:space="preserve">   to a planting pattern that keeps the cooler under its ceiling — an answer v4 could not</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   even represent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>WHAT v5 STILL DOES NOT CARRY</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Costs are seed/transplant per acre ONLY: no labour, water, packaging, storage, overhead.</t>
+          <t xml:space="preserve">   even represent.</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Profit is therefore far too high. The cash layer is next.</t>
-        </is>
-      </c>
+      <c r="A118" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - No cash-flow constraint, so it can spend money it does not have.</t>
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>WHAT v5 STILL DOES NOT CARRY</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Shelf life IS enforced now (a real constraint since you found it dead). Shrink is wired</t>
+          <t xml:space="preserve">  - Costs are seed/transplant per acre ONLY: no labour, water, packaging, storage, overhead.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">    too, but defaults to 0%, so it stays invisible until you set it.</t>
+          <t xml:space="preserve">    Profit is therefore far too high. The cash layer is next.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - No water, labour, diversity or throughput limits.</t>
+          <t xml:space="preserve">  - No cash-flow constraint, so it can spend money it does not have.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Three crops, not seven.</t>
+          <t xml:space="preserve">  - Shelf life IS enforced now (a real constraint since you found it dead). Shrink is wired</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
+      <c r="A124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    too, but defaults to 0%, so it stays invisible until you set it.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="inlineStr">
-        <is>
-          <t>!! THE SCALE WARNING</t>
+      <c r="A125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - No water, labour, diversity or throughput limits.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Three crops, not seven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>!! THE SCALE WARNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
           <t>An optimizer's answer is far more scale-sensitive than a calculator's: which constraint binds,</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
+    <row r="130">
+      <c r="A130" t="inlineStr">
         <is>
           <t>and therefore which crop and which WEEK wins, can invert between 3 crops and 7. This teaches</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>the machinery. It is not advice about your farm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>HAS THIS SHEET BEEN CHECKED?</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Yes. Crop data, the calendar and the demand caps are read from the app. The formulas are</t>
+          <t>the machinery. It is not advice about your farm.</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>calculated by an engine and compared cell by cell against an independent model under three</t>
-        </is>
-      </c>
+      <c r="A132" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>configurations. Every input is perturbed to prove it propagates. No number is frozen. And the</t>
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>HAS THIS SHEET BEEN CHECKED?</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>same MILP is solved with scipy.milp, its answer written into the decision cells, and the</t>
+          <t>Yes. Crop data, the calendar and the demand caps are read from the app. The formulas are</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>sheet's own PROFIT cell must reproduce the optimum exactly.</t>
+          <t>calculated by an engine and compared cell by cell against an independent model under three</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
+        <is>
+          <t>configurations. Every input is perturbed to prove it propagates. No number is frozen. And the</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>same MILP is solved with scipy.milp, its answer written into the decision cells, and the</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>sheet's own PROFIT cell must reproduce the optimum exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
         <is>
           <t xml:space="preserve">     Run it yourself:   .venv/bin/python toy_models/verify_toy_v5.py</t>
         </is>
@@ -1509,23 +1530,28 @@
           <t>FARM TOY MODEL — v5: the full calendar (a MILP)</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>BUILT 2026-08-30 13:25   (from source at a6c69e1)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>YELLOW = you type.  GREEN = the solver writes.  BLUE = the solver's plant/don't-plant switches.  Read the 'READ ME' sheet first.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>1 — THE FARM</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Land you have</t>
         </is>
@@ -1533,14 +1559,14 @@
       <c r="B5" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>acres</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Cold store (cooler)</t>
         </is>
@@ -1548,14 +1574,14 @@
       <c r="B6" s="6" t="n">
         <v>275</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>m3 — Spinach, Kale</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Ambient store (barn)</t>
         </is>
@@ -1563,14 +1589,14 @@
       <c r="B7" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>m3 — Garlic</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>2 — HOW EACH CROP BEHAVES</t>
         </is>
@@ -1723,14 +1749,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>'Min acres if planted' is what the plant/don't-plant switch enforces — see section 4.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>3 — WHO BUYS IT   (one row per crop x channel — the grower's ruling)</t>
         </is>
@@ -1994,14 +2020,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>4 — THE PLANTING CALENDAR   (68 possible plantings — the solver picks)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>One row per legal start week, exactly what the app's generator offers. ACRES and PLANT? are both decisions.</t>
         </is>
@@ -8131,7 +8157,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>ACRES &lt;= 'max if planted' and ACRES &gt;= 'min if planted' are the app's C9 and C10: you cannot plant acres without deciding to plant, and if you plant at all you plant a real block.</t>
         </is>
@@ -8306,12 +8332,12 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="3" t="inlineStr">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t>LAND in the ground</t>
         </is>
       </c>
-      <c r="B99" s="4" t="inlineStr">
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t>used</t>
         </is>
@@ -8526,7 +8552,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="3" t="inlineStr"/>
+      <c r="A100" s="4" t="inlineStr"/>
       <c r="E100" s="32" t="inlineStr">
         <is>
           <t>&lt;=</t>
@@ -8789,12 +8815,12 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="3" t="inlineStr">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  limit</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
+      <c r="B101" s="2" t="inlineStr">
         <is>
           <t>cap</t>
         </is>
@@ -9224,14 +9250,14 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="inlineStr">
+      <c r="A103" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Acres standing that week, summed across every planting the solver chose.</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="inlineStr">
+      <c r="A105" s="3" t="inlineStr">
         <is>
           <t>SPINACH  —  cold store</t>
         </is>
@@ -9403,12 +9429,12 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="3" t="inlineStr">
+      <c r="A107" s="4" t="inlineStr">
         <is>
           <t>Packed out -&gt; INTO the store</t>
         </is>
       </c>
-      <c r="B107" s="4" t="inlineStr">
+      <c r="B107" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -9628,7 +9654,7 @@
           <t>Stock carried in</t>
         </is>
       </c>
-      <c r="B108" s="4" t="inlineStr">
+      <c r="B108" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -9847,7 +9873,7 @@
           <t xml:space="preserve">   lost to shrink</t>
         </is>
       </c>
-      <c r="B109" s="4" t="inlineStr">
+      <c r="B109" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -10062,12 +10088,12 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="inlineStr">
+      <c r="A110" s="4" t="inlineStr">
         <is>
           <t>In store this week</t>
         </is>
       </c>
-      <c r="B110" s="4" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -10287,7 +10313,7 @@
           <t>Farmers Market — most you may sell this week</t>
         </is>
       </c>
-      <c r="B111" s="4" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -10507,7 +10533,7 @@
           <t>Farmers Market — OFFERED</t>
         </is>
       </c>
-      <c r="B112" s="4" t="inlineStr">
+      <c r="B112" s="2" t="inlineStr">
         <is>
           <t>lb  &lt;-- SOLVER</t>
         </is>
@@ -10675,7 +10701,7 @@
           <t>Farmers Market — SOLD</t>
         </is>
       </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -10895,7 +10921,7 @@
           <t xml:space="preserve">   market loss (gone)</t>
         </is>
       </c>
-      <c r="B114" s="4" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -11115,7 +11141,7 @@
           <t xml:space="preserve">   returned to store</t>
         </is>
       </c>
-      <c r="B115" s="4" t="inlineStr">
+      <c r="B115" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -11335,7 +11361,7 @@
           <t xml:space="preserve">   leaves the store (offered - returned)</t>
         </is>
       </c>
-      <c r="B116" s="4" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -11555,7 +11581,7 @@
           <t>Wholesale — most you may sell this week</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -11775,7 +11801,7 @@
           <t>Wholesale — OFFERED</t>
         </is>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t>lb  &lt;-- SOLVER</t>
         </is>
@@ -11943,7 +11969,7 @@
           <t>Wholesale — SOLD</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -12163,7 +12189,7 @@
           <t xml:space="preserve">   market loss (gone)</t>
         </is>
       </c>
-      <c r="B120" s="4" t="inlineStr">
+      <c r="B120" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -12383,7 +12409,7 @@
           <t xml:space="preserve">   returned to store</t>
         </is>
       </c>
-      <c r="B121" s="4" t="inlineStr">
+      <c r="B121" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -12603,7 +12629,7 @@
           <t xml:space="preserve">   leaves the store (offered - returned)</t>
         </is>
       </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -12818,12 +12844,12 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="3" t="inlineStr">
+      <c r="A123" s="4" t="inlineStr">
         <is>
           <t>Stock carried out</t>
         </is>
       </c>
-      <c r="B123" s="4" t="inlineStr">
+      <c r="B123" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -13038,14 +13064,14 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="4" t="inlineStr">
+      <c r="A124" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   ^ subtracts what LEAVES, not what was offered — so 'returned to store' is</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="4" t="inlineStr">
+      <c r="A125" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">     never taken out at all, and shows up as next week's carried in.</t>
         </is>
@@ -13057,7 +13083,7 @@
           <t>Most stock its shelf life allows</t>
         </is>
       </c>
-      <c r="B126" s="4" t="inlineStr">
+      <c r="B126" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -13272,19 +13298,19 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="4" t="inlineStr">
+      <c r="A127" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Stock carried out must stay at or below this row.</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="3" t="inlineStr">
+      <c r="A128" s="4" t="inlineStr">
         <is>
           <t>ROOM OCCUPANCY</t>
         </is>
       </c>
-      <c r="B128" s="4" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
@@ -13499,7 +13525,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="inlineStr">
+      <c r="A130" s="3" t="inlineStr">
         <is>
           <t>KALE  —  cold store</t>
         </is>
@@ -13671,12 +13697,12 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="3" t="inlineStr">
+      <c r="A132" s="4" t="inlineStr">
         <is>
           <t>Packed out -&gt; INTO the store</t>
         </is>
       </c>
-      <c r="B132" s="4" t="inlineStr">
+      <c r="B132" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -13896,7 +13922,7 @@
           <t>Stock carried in</t>
         </is>
       </c>
-      <c r="B133" s="4" t="inlineStr">
+      <c r="B133" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -14115,7 +14141,7 @@
           <t xml:space="preserve">   lost to shrink</t>
         </is>
       </c>
-      <c r="B134" s="4" t="inlineStr">
+      <c r="B134" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -14330,12 +14356,12 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="3" t="inlineStr">
+      <c r="A135" s="4" t="inlineStr">
         <is>
           <t>In store this week</t>
         </is>
       </c>
-      <c r="B135" s="4" t="inlineStr">
+      <c r="B135" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -14555,7 +14581,7 @@
           <t>Farmers Market — most you may sell this week</t>
         </is>
       </c>
-      <c r="B136" s="4" t="inlineStr">
+      <c r="B136" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -14775,7 +14801,7 @@
           <t>Farmers Market — OFFERED</t>
         </is>
       </c>
-      <c r="B137" s="4" t="inlineStr">
+      <c r="B137" s="2" t="inlineStr">
         <is>
           <t>lb  &lt;-- SOLVER</t>
         </is>
@@ -14943,7 +14969,7 @@
           <t>Farmers Market — SOLD</t>
         </is>
       </c>
-      <c r="B138" s="4" t="inlineStr">
+      <c r="B138" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -15163,7 +15189,7 @@
           <t xml:space="preserve">   market loss (gone)</t>
         </is>
       </c>
-      <c r="B139" s="4" t="inlineStr">
+      <c r="B139" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -15383,7 +15409,7 @@
           <t xml:space="preserve">   returned to store</t>
         </is>
       </c>
-      <c r="B140" s="4" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -15603,7 +15629,7 @@
           <t xml:space="preserve">   leaves the store (offered - returned)</t>
         </is>
       </c>
-      <c r="B141" s="4" t="inlineStr">
+      <c r="B141" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -15823,7 +15849,7 @@
           <t>Wholesale — most you may sell this week</t>
         </is>
       </c>
-      <c r="B142" s="4" t="inlineStr">
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -16038,14 +16064,14 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="4" t="inlineStr">
+      <c r="A143" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   ^ Wholesale is an ANNUAL cap (500,000 lb a year), so there is NO weekly limit —</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="4" t="inlineStr">
+      <c r="A144" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">     this row is what is LEFT of the year, and it falls as you sell.</t>
         </is>
@@ -16057,7 +16083,7 @@
           <t>Wholesale — OFFERED</t>
         </is>
       </c>
-      <c r="B145" s="4" t="inlineStr">
+      <c r="B145" s="2" t="inlineStr">
         <is>
           <t>lb  &lt;-- SOLVER</t>
         </is>
@@ -16225,7 +16251,7 @@
           <t>Wholesale — SOLD</t>
         </is>
       </c>
-      <c r="B146" s="4" t="inlineStr">
+      <c r="B146" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -16445,7 +16471,7 @@
           <t xml:space="preserve">   market loss (gone)</t>
         </is>
       </c>
-      <c r="B147" s="4" t="inlineStr">
+      <c r="B147" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -16665,7 +16691,7 @@
           <t xml:space="preserve">   returned to store</t>
         </is>
       </c>
-      <c r="B148" s="4" t="inlineStr">
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -16885,7 +16911,7 @@
           <t xml:space="preserve">   leaves the store (offered - returned)</t>
         </is>
       </c>
-      <c r="B149" s="4" t="inlineStr">
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -17100,12 +17126,12 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="3" t="inlineStr">
+      <c r="A150" s="4" t="inlineStr">
         <is>
           <t>Stock carried out</t>
         </is>
       </c>
-      <c r="B150" s="4" t="inlineStr">
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -17320,14 +17346,14 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="4" t="inlineStr">
+      <c r="A151" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   ^ subtracts what LEAVES, not what was offered — so 'returned to store' is</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="4" t="inlineStr">
+      <c r="A152" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">     never taken out at all, and shows up as next week's carried in.</t>
         </is>
@@ -17339,7 +17365,7 @@
           <t>Most stock its shelf life allows</t>
         </is>
       </c>
-      <c r="B153" s="4" t="inlineStr">
+      <c r="B153" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -17554,19 +17580,19 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="4" t="inlineStr">
+      <c r="A154" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Stock carried out must stay at or below this row.</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="3" t="inlineStr">
+      <c r="A155" s="4" t="inlineStr">
         <is>
           <t>ROOM OCCUPANCY</t>
         </is>
       </c>
-      <c r="B155" s="4" t="inlineStr">
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
@@ -17781,7 +17807,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="inlineStr">
+      <c r="A157" s="3" t="inlineStr">
         <is>
           <t>GARLIC  —  ambient store</t>
         </is>
@@ -17953,12 +17979,12 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="3" t="inlineStr">
+      <c r="A159" s="4" t="inlineStr">
         <is>
           <t>Packed out -&gt; INTO the store</t>
         </is>
       </c>
-      <c r="B159" s="4" t="inlineStr">
+      <c r="B159" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -18178,7 +18204,7 @@
           <t>Stock carried in</t>
         </is>
       </c>
-      <c r="B160" s="4" t="inlineStr">
+      <c r="B160" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -18397,7 +18423,7 @@
           <t xml:space="preserve">   lost to shrink</t>
         </is>
       </c>
-      <c r="B161" s="4" t="inlineStr">
+      <c r="B161" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -18612,12 +18638,12 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="3" t="inlineStr">
+      <c r="A162" s="4" t="inlineStr">
         <is>
           <t>In store this week</t>
         </is>
       </c>
-      <c r="B162" s="4" t="inlineStr">
+      <c r="B162" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -18837,7 +18863,7 @@
           <t>Farmers Market — most you may sell this week</t>
         </is>
       </c>
-      <c r="B163" s="4" t="inlineStr">
+      <c r="B163" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -19057,7 +19083,7 @@
           <t>Farmers Market — OFFERED</t>
         </is>
       </c>
-      <c r="B164" s="4" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
         <is>
           <t>lb  &lt;-- SOLVER</t>
         </is>
@@ -19225,7 +19251,7 @@
           <t>Farmers Market — SOLD</t>
         </is>
       </c>
-      <c r="B165" s="4" t="inlineStr">
+      <c r="B165" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -19445,7 +19471,7 @@
           <t xml:space="preserve">   market loss (gone)</t>
         </is>
       </c>
-      <c r="B166" s="4" t="inlineStr">
+      <c r="B166" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -19665,7 +19691,7 @@
           <t xml:space="preserve">   returned to store</t>
         </is>
       </c>
-      <c r="B167" s="4" t="inlineStr">
+      <c r="B167" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -19885,7 +19911,7 @@
           <t xml:space="preserve">   leaves the store (offered - returned)</t>
         </is>
       </c>
-      <c r="B168" s="4" t="inlineStr">
+      <c r="B168" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -20105,7 +20131,7 @@
           <t>Wholesale — most you may sell this week</t>
         </is>
       </c>
-      <c r="B169" s="4" t="inlineStr">
+      <c r="B169" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -20325,7 +20351,7 @@
           <t>Wholesale — OFFERED</t>
         </is>
       </c>
-      <c r="B170" s="4" t="inlineStr">
+      <c r="B170" s="2" t="inlineStr">
         <is>
           <t>lb  &lt;-- SOLVER</t>
         </is>
@@ -20493,7 +20519,7 @@
           <t>Wholesale — SOLD</t>
         </is>
       </c>
-      <c r="B171" s="4" t="inlineStr">
+      <c r="B171" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -20713,7 +20739,7 @@
           <t xml:space="preserve">   market loss (gone)</t>
         </is>
       </c>
-      <c r="B172" s="4" t="inlineStr">
+      <c r="B172" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -20933,7 +20959,7 @@
           <t xml:space="preserve">   returned to store</t>
         </is>
       </c>
-      <c r="B173" s="4" t="inlineStr">
+      <c r="B173" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -21153,7 +21179,7 @@
           <t xml:space="preserve">   leaves the store (offered - returned)</t>
         </is>
       </c>
-      <c r="B174" s="4" t="inlineStr">
+      <c r="B174" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -21368,12 +21394,12 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="3" t="inlineStr">
+      <c r="A175" s="4" t="inlineStr">
         <is>
           <t>Stock carried out</t>
         </is>
       </c>
-      <c r="B175" s="4" t="inlineStr">
+      <c r="B175" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -21588,14 +21614,14 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="4" t="inlineStr">
+      <c r="A176" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   ^ subtracts what LEAVES, not what was offered — so 'returned to store' is</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="4" t="inlineStr">
+      <c r="A177" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">     never taken out at all, and shows up as next week's carried in.</t>
         </is>
@@ -21607,7 +21633,7 @@
           <t>Most stock its shelf life allows</t>
         </is>
       </c>
-      <c r="B178" s="4" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
@@ -21822,19 +21848,19 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="4" t="inlineStr">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Stock carried out must stay at or below this row.</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="3" t="inlineStr">
+      <c r="A180" s="4" t="inlineStr">
         <is>
           <t>ROOM OCCUPANCY</t>
         </is>
       </c>
-      <c r="B180" s="4" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
@@ -22049,7 +22075,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+      <c r="A182" s="3" t="inlineStr">
         <is>
           <t>6 — THE TWO STORES</t>
         </is>
@@ -22229,7 +22255,7 @@
           <t>COLD STORE</t>
         </is>
       </c>
-      <c r="B184" s="4" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>used</t>
         </is>
@@ -22444,7 +22470,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="3" t="inlineStr"/>
+      <c r="A185" s="4" t="inlineStr"/>
       <c r="E185" s="32" t="inlineStr">
         <is>
           <t>&lt;=</t>
@@ -22707,12 +22733,12 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="3" t="inlineStr">
+      <c r="A186" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  limit</t>
         </is>
       </c>
-      <c r="B186" s="4" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>cap</t>
         </is>
@@ -23142,7 +23168,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="4" t="inlineStr">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Holds Spinach, Kale.</t>
         </is>
@@ -23322,7 +23348,7 @@
           <t>AMBIENT STORE</t>
         </is>
       </c>
-      <c r="B191" s="4" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>used</t>
         </is>
@@ -23537,7 +23563,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="3" t="inlineStr"/>
+      <c r="A192" s="4" t="inlineStr"/>
       <c r="E192" s="32" t="inlineStr">
         <is>
           <t>&lt;=</t>
@@ -23800,12 +23826,12 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="3" t="inlineStr">
+      <c r="A193" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  limit</t>
         </is>
       </c>
-      <c r="B193" s="4" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>cap</t>
         </is>
@@ -24235,21 +24261,21 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="4" t="inlineStr">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Holds Garlic.</t>
         </is>
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="inlineStr">
+      <c r="A197" s="3" t="inlineStr">
         <is>
           <t>7 — THE OPTIMIZER</t>
         </is>
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="3" t="inlineStr">
+      <c r="A198" s="4" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
@@ -24260,7 +24286,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="3" t="inlineStr">
+      <c r="A199" s="4" t="inlineStr">
         <is>
           <t>Growing cost</t>
         </is>
@@ -24269,7 +24295,7 @@
         <f>SUMPRODUCT($C$28:$C$95,($B$28:$B$95="Spinach")*$H$11+($B$28:$B$95="Kale")*$H$12+($B$28:$B$95="Garlic")*$H$13)</f>
         <v/>
       </c>
-      <c r="C199" s="4" t="inlineStr">
+      <c r="C199" s="2" t="inlineStr">
         <is>
           <t>acres x $/acre, across every planting</t>
         </is>
@@ -24285,14 +24311,14 @@
         <f>B198-B199</f>
         <v/>
       </c>
-      <c r="C200" s="3" t="inlineStr">
+      <c r="C200" s="4" t="inlineStr">
         <is>
           <t>&lt;-- MAXIMISE THIS CELL</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="3" t="inlineStr">
+      <c r="A201" s="4" t="inlineStr">
         <is>
           <t>Plantings chosen</t>
         </is>
@@ -24301,14 +24327,14 @@
         <f>SUM($D$28:$D$95)</f>
         <v/>
       </c>
-      <c r="C201" s="4" t="inlineStr">
+      <c r="C201" s="2" t="inlineStr">
         <is>
           <t>of 68 offered</t>
         </is>
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="3" t="inlineStr">
+      <c r="A203" s="4" t="inlineStr">
         <is>
           <t>Annual caps</t>
         </is>
@@ -24335,14 +24361,14 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="inlineStr">
+      <c r="A206" s="3" t="inlineStr">
         <is>
           <t>SOLVER SETUP — Tools &gt; Solver</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="3" t="inlineStr">
+      <c r="A207" s="4" t="inlineStr">
         <is>
           <t>Target cell</t>
         </is>
@@ -24352,14 +24378,14 @@
           <t>$B$200</t>
         </is>
       </c>
-      <c r="G207" s="4" t="inlineStr">
+      <c r="G207" s="2" t="inlineStr">
         <is>
           <t>set to MAXIMUM</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="3" t="inlineStr">
+      <c r="A208" s="4" t="inlineStr">
         <is>
           <t>By changing cells</t>
         </is>
@@ -24369,7 +24395,7 @@
           <t>$C$28:$D$95</t>
         </is>
       </c>
-      <c r="G208" s="4" t="inlineStr">
+      <c r="G208" s="2" t="inlineStr">
         <is>
           <t>acres AND plant? together</t>
         </is>
@@ -24386,7 +24412,7 @@
           <t>$E$112:$BD$112;$E$118:$BD$118;$E$137:$BD$137;$E$145:$BD$145;$E$164:$BD$164;$E$170:$BD$170</t>
         </is>
       </c>
-      <c r="G209" s="4" t="inlineStr">
+      <c r="G209" s="2" t="inlineStr">
         <is>
           <t>the OFFERED rows</t>
         </is>
@@ -24415,7 +24441,7 @@
           <t>$C$28:$C$95  &lt;=  $BE$28:$BE$95</t>
         </is>
       </c>
-      <c r="G211" s="4" t="inlineStr">
+      <c r="G211" s="2" t="inlineStr">
         <is>
           <t>no acres without deciding to plant</t>
         </is>
@@ -24432,7 +24458,7 @@
           <t>$C$28:$C$95  &gt;=  $BF$28:$BF$95</t>
         </is>
       </c>
-      <c r="G212" s="4" t="inlineStr">
+      <c r="G212" s="2" t="inlineStr">
         <is>
           <t>planted means a real block</t>
         </is>
@@ -24557,7 +24583,7 @@
           <t>$E$123:$BD$123  &lt;=  $E$126:$BD$126</t>
         </is>
       </c>
-      <c r="G222" s="4" t="inlineStr">
+      <c r="G222" s="2" t="inlineStr">
         <is>
           <t>nothing held longer than it keeps</t>
         </is>
@@ -24574,7 +24600,7 @@
           <t>$E$150:$BD$150  &lt;=  $E$153:$BD$153</t>
         </is>
       </c>
-      <c r="G223" s="4" t="inlineStr">
+      <c r="G223" s="2" t="inlineStr">
         <is>
           <t>nothing held longer than it keeps</t>
         </is>
@@ -24591,7 +24617,7 @@
           <t>$E$175:$BD$175  &lt;=  $E$178:$BD$178</t>
         </is>
       </c>
-      <c r="G224" s="4" t="inlineStr">
+      <c r="G224" s="2" t="inlineStr">
         <is>
           <t>nothing held longer than it keeps</t>
         </is>
@@ -24634,7 +24660,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="3" t="inlineStr">
+      <c r="A228" s="4" t="inlineStr">
         <is>
           <t>Options</t>
         </is>
@@ -24644,7 +24670,7 @@
           <t>engine = LibreOffice CoinMP Linear Solver</t>
         </is>
       </c>
-      <c r="G228" s="4" t="inlineStr">
+      <c r="G228" s="2" t="inlineStr">
         <is>
           <t>tick 'Assume variables as non-negative'</t>
         </is>

</xml_diff>